<commit_message>
update import and export
</commit_message>
<xml_diff>
--- a/example/HoGiaDinh_Import_Template.xlsx
+++ b/example/HoGiaDinh_Import_Template.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import_HoGiaDinh" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HoGiaDinh" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NhanKhau" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +26,24 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +58,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,128 +428,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Số căn hộ</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Chủ hộ</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Tầng / Khu vực</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Diện tích</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>soCanHo (*)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>chuHo (*)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tangKhuVuc</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dienTich_m2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ghiChu</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>101</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Nguyen Van A</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Tầng 1</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>75.5</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>a@gmail.com</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Hộ mẫu 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>102</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Tran Thi B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Tầng 1</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>80</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>b@gmail.com</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Hộ mẫu 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>103</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Le Van C</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Tầng 1</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>65</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>c@gmail.com</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Hộ mẫu 3</t>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>hoTen (*)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ngaySinh (dd/MM/yyyy)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>gioiTinh</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>cccd</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>soDienThoai</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>quanHeChuHo</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>soCanHo (*)</t>
         </is>
       </c>
     </row>

</xml_diff>